<commit_message>
refactor: generalize telecom domain, add seed datasets and clean architecture specs
</commit_message>
<xml_diff>
--- a/data/Reporte_Gerencial_Facturacion_Estilizado.xlsx
+++ b/data/Reporte_Gerencial_Facturacion_Estilizado.xlsx
@@ -70,8 +70,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DA291C"/>
-        <bgColor rgb="00DA291C"/>
+        <fgColor rgb="00005A9E"/>
+        <bgColor rgb="00005A9E"/>
       </patternFill>
     </fill>
     <fill>
@@ -519,7 +519,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CLARO PERÚ — REPORTE OPERACIONAL DE POST FACTURACIÓN (Resumen KPIs)</t>
+          <t>TELECOM ENTERPRISE — REPORTE OPERACIONAL DE POST FACTURACIÓN (Resumen KPIs)</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CLARO PERÚ — REPORTE OPERACIONAL DE POST FACTURACIÓN (Detalle Ciclos)</t>
+          <t>TELECOM ENTERPRISE — REPORTE OPERACIONAL DE POST FACTURACIÓN (Detalle Ciclos)</t>
         </is>
       </c>
     </row>

</xml_diff>